<commit_message>
Fix Day 6 topic index resolution and identical topic name mapping
</commit_message>
<xml_diff>
--- a/outputs/filled_feedback_0d9db05d.xlsx
+++ b/outputs/filled_feedback_0d9db05d.xlsx
@@ -1795,7 +1795,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
               </a:p>
             </txPr>
@@ -1902,7 +1902,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
           </a:p>
         </txPr>
@@ -1940,7 +1940,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
           </a:p>
         </txPr>
@@ -2340,7 +2340,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X88"/>
+  <dimension ref="A1:Z87"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col width="16.1238095238095" customWidth="1" style="70" min="1" max="1"/>
@@ -2368,8 +2368,8 @@
       <c r="N1" s="34" t="n"/>
       <c r="O1" s="34" t="n"/>
       <c r="P1" s="34" t="n"/>
-      <c r="V1" s="35" t="n"/>
-      <c r="W1" s="36" t="n"/>
+      <c r="X1" s="35" t="n"/>
+      <c r="Y1" s="36" t="n"/>
     </row>
     <row r="2" ht="26.25" customHeight="1" s="70">
       <c r="A2" s="37" t="n"/>
@@ -2397,8 +2397,10 @@
       <c r="N2" s="86" t="n"/>
       <c r="O2" s="86" t="n"/>
       <c r="P2" s="86" t="n"/>
-      <c r="V2" s="86" t="n"/>
-      <c r="W2" s="87" t="n"/>
+      <c r="Q2" s="86" t="n"/>
+      <c r="R2" s="87" t="n"/>
+      <c r="X2" s="86" t="n"/>
+      <c r="Y2" s="87" t="n"/>
     </row>
     <row r="3" ht="18" customHeight="1" s="70">
       <c r="A3" s="40" t="n"/>
@@ -2429,8 +2431,10 @@
       <c r="N3" s="86" t="n"/>
       <c r="O3" s="86" t="n"/>
       <c r="P3" s="86" t="n"/>
-      <c r="V3" s="86" t="n"/>
-      <c r="W3" s="87" t="n"/>
+      <c r="Q3" s="86" t="n"/>
+      <c r="R3" s="87" t="n"/>
+      <c r="X3" s="86" t="n"/>
+      <c r="Y3" s="87" t="n"/>
     </row>
     <row r="4" ht="18" customHeight="1" s="70">
       <c r="A4" s="43" t="inlineStr">
@@ -2466,12 +2470,12 @@
       <c r="N4" s="86" t="n"/>
       <c r="O4" s="86" t="n"/>
       <c r="P4" s="87" t="n"/>
-      <c r="V4" s="46" t="inlineStr">
+      <c r="X4" s="46" t="inlineStr">
         <is>
           <t>Avg</t>
         </is>
       </c>
-      <c r="W4" s="44" t="inlineStr">
+      <c r="Y4" s="44" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
@@ -2524,33 +2528,33 @@
       <c r="P5" s="53" t="n">
         <v>212856</v>
       </c>
-      <c r="Q5" t="inlineStr">
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>E 211/27</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>E213580</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>210771</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
         <is>
           <t>213328</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
+      <c r="W5" t="inlineStr">
         <is>
           <t>8213570</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>E 211/27</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>E213580</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>210771</t>
-        </is>
-      </c>
-      <c r="V5" s="88" t="n"/>
-      <c r="W5" s="88" t="n"/>
+      <c r="X5" s="88" t="n"/>
+      <c r="Y5" s="88" t="n"/>
     </row>
     <row r="6" ht="19.5" customHeight="1" s="70">
       <c r="A6" s="48" t="inlineStr">
@@ -2614,8 +2618,14 @@
       <c r="U6" t="n">
         <v>10</v>
       </c>
-      <c r="V6" s="89" t="n"/>
-      <c r="W6" s="41" t="n"/>
+      <c r="V6" t="n">
+        <v>10</v>
+      </c>
+      <c r="W6" t="n">
+        <v>9</v>
+      </c>
+      <c r="X6" s="89" t="n"/>
+      <c r="Y6" s="41" t="n"/>
     </row>
     <row r="7" ht="19.5" customHeight="1" s="70">
       <c r="A7" s="90" t="n"/>
@@ -2669,8 +2679,14 @@
       <c r="U7" t="n">
         <v>10</v>
       </c>
-      <c r="V7" s="89" t="n"/>
-      <c r="W7" s="41" t="n"/>
+      <c r="V7" t="n">
+        <v>9</v>
+      </c>
+      <c r="W7" t="n">
+        <v>9</v>
+      </c>
+      <c r="X7" s="89" t="n"/>
+      <c r="Y7" s="41" t="n"/>
     </row>
     <row r="8" ht="19.5" customHeight="1" s="70">
       <c r="A8" s="90" t="n"/>
@@ -2724,8 +2740,14 @@
       <c r="U8" t="n">
         <v>10</v>
       </c>
-      <c r="V8" s="89" t="n"/>
-      <c r="W8" s="41" t="n"/>
+      <c r="V8" t="n">
+        <v>9</v>
+      </c>
+      <c r="W8" t="n">
+        <v>7</v>
+      </c>
+      <c r="X8" s="89" t="n"/>
+      <c r="Y8" s="41" t="n"/>
     </row>
     <row r="9" ht="19.5" customHeight="1" s="70">
       <c r="A9" s="90" t="n"/>
@@ -2779,8 +2801,14 @@
       <c r="U9" t="n">
         <v>10</v>
       </c>
-      <c r="V9" s="89" t="n"/>
-      <c r="W9" s="41" t="n"/>
+      <c r="V9" t="n">
+        <v>9</v>
+      </c>
+      <c r="W9" t="n">
+        <v>9</v>
+      </c>
+      <c r="X9" s="89" t="n"/>
+      <c r="Y9" s="41" t="n"/>
     </row>
     <row r="10" ht="19.5" customHeight="1" s="70">
       <c r="A10" s="90" t="n"/>
@@ -2834,8 +2862,14 @@
       <c r="U10" t="n">
         <v>10</v>
       </c>
-      <c r="V10" s="89" t="n"/>
-      <c r="W10" s="41" t="n"/>
+      <c r="V10" t="n">
+        <v>9</v>
+      </c>
+      <c r="W10" t="n">
+        <v>9</v>
+      </c>
+      <c r="X10" s="89" t="n"/>
+      <c r="Y10" s="41" t="n"/>
     </row>
     <row r="11" ht="19.5" customHeight="1" s="70">
       <c r="A11" s="90" t="n"/>
@@ -2894,8 +2928,14 @@
       <c r="U11" t="n">
         <v>10</v>
       </c>
-      <c r="V11" s="89" t="n"/>
-      <c r="W11" s="41" t="n"/>
+      <c r="V11" t="n">
+        <v>10</v>
+      </c>
+      <c r="W11" t="n">
+        <v>10</v>
+      </c>
+      <c r="X11" s="89" t="n"/>
+      <c r="Y11" s="41" t="n"/>
     </row>
     <row r="12" ht="19.5" customHeight="1" s="70">
       <c r="A12" s="90" t="n"/>
@@ -2949,8 +2989,14 @@
       <c r="U12" t="n">
         <v>10</v>
       </c>
-      <c r="V12" s="89" t="n"/>
-      <c r="W12" s="41" t="n"/>
+      <c r="V12" t="n">
+        <v>9</v>
+      </c>
+      <c r="W12" t="n">
+        <v>10</v>
+      </c>
+      <c r="X12" s="89" t="n"/>
+      <c r="Y12" s="41" t="n"/>
     </row>
     <row r="13" ht="19.5" customHeight="1" s="70">
       <c r="A13" s="90" t="n"/>
@@ -3004,8 +3050,14 @@
       <c r="U13" t="n">
         <v>10</v>
       </c>
-      <c r="V13" s="89" t="n"/>
-      <c r="W13" s="41" t="n"/>
+      <c r="V13" t="n">
+        <v>9</v>
+      </c>
+      <c r="W13" t="n">
+        <v>10</v>
+      </c>
+      <c r="X13" s="89" t="n"/>
+      <c r="Y13" s="41" t="n"/>
     </row>
     <row r="14" ht="19.5" customHeight="1" s="70">
       <c r="A14" s="90" t="n"/>
@@ -3059,8 +3111,14 @@
       <c r="U14" t="n">
         <v>10</v>
       </c>
-      <c r="V14" s="89" t="n"/>
-      <c r="W14" s="41" t="n"/>
+      <c r="V14" t="n">
+        <v>9</v>
+      </c>
+      <c r="W14" t="n">
+        <v>10</v>
+      </c>
+      <c r="X14" s="89" t="n"/>
+      <c r="Y14" s="41" t="n"/>
     </row>
     <row r="15" ht="19.5" customHeight="1" s="70">
       <c r="A15" s="88" t="n"/>
@@ -3114,8 +3172,14 @@
       <c r="U15" t="n">
         <v>10</v>
       </c>
-      <c r="V15" s="89" t="n"/>
-      <c r="W15" s="41" t="n"/>
+      <c r="V15" t="n">
+        <v>9</v>
+      </c>
+      <c r="W15" t="n">
+        <v>10</v>
+      </c>
+      <c r="X15" s="89" t="n"/>
+      <c r="Y15" s="41" t="n"/>
     </row>
     <row r="16" ht="19.5" customHeight="1" s="70">
       <c r="A16" s="48" t="inlineStr">
@@ -3179,8 +3243,14 @@
       <c r="U16" t="n">
         <v>10</v>
       </c>
-      <c r="V16" s="89" t="n"/>
-      <c r="W16" s="41" t="n"/>
+      <c r="V16" t="n">
+        <v>10</v>
+      </c>
+      <c r="W16" t="n">
+        <v>10</v>
+      </c>
+      <c r="X16" s="89" t="n"/>
+      <c r="Y16" s="41" t="n"/>
     </row>
     <row r="17" ht="19.5" customHeight="1" s="70">
       <c r="A17" s="90" t="n"/>
@@ -3234,8 +3304,14 @@
       <c r="U17" t="n">
         <v>10</v>
       </c>
-      <c r="V17" s="89" t="n"/>
-      <c r="W17" s="41" t="n"/>
+      <c r="V17" t="n">
+        <v>9</v>
+      </c>
+      <c r="W17" t="n">
+        <v>10</v>
+      </c>
+      <c r="X17" s="89" t="n"/>
+      <c r="Y17" s="41" t="n"/>
     </row>
     <row r="18" ht="19.5" customHeight="1" s="70">
       <c r="A18" s="90" t="n"/>
@@ -3289,8 +3365,14 @@
       <c r="U18" t="n">
         <v>10</v>
       </c>
-      <c r="V18" s="89" t="n"/>
-      <c r="W18" s="41" t="n"/>
+      <c r="V18" t="n">
+        <v>9</v>
+      </c>
+      <c r="W18" t="n">
+        <v>10</v>
+      </c>
+      <c r="X18" s="89" t="n"/>
+      <c r="Y18" s="41" t="n"/>
     </row>
     <row r="19" ht="19.5" customHeight="1" s="70">
       <c r="A19" s="90" t="n"/>
@@ -3344,8 +3426,14 @@
       <c r="U19" t="n">
         <v>10</v>
       </c>
-      <c r="V19" s="89" t="n"/>
-      <c r="W19" s="41" t="n"/>
+      <c r="V19" t="n">
+        <v>9</v>
+      </c>
+      <c r="W19" t="n">
+        <v>10</v>
+      </c>
+      <c r="X19" s="89" t="n"/>
+      <c r="Y19" s="41" t="n"/>
     </row>
     <row r="20" ht="19.5" customHeight="1" s="70">
       <c r="A20" s="90" t="n"/>
@@ -3399,8 +3487,14 @@
       <c r="U20" t="n">
         <v>10</v>
       </c>
-      <c r="V20" s="89" t="n"/>
-      <c r="W20" s="41" t="n"/>
+      <c r="V20" t="n">
+        <v>9</v>
+      </c>
+      <c r="W20" t="n">
+        <v>10</v>
+      </c>
+      <c r="X20" s="89" t="n"/>
+      <c r="Y20" s="41" t="n"/>
     </row>
     <row r="21" ht="19.5" customHeight="1" s="70">
       <c r="A21" s="90" t="n"/>
@@ -3459,8 +3553,14 @@
       <c r="U21" t="n">
         <v>10</v>
       </c>
-      <c r="V21" s="89" t="n"/>
-      <c r="W21" s="41" t="n"/>
+      <c r="V21" t="n">
+        <v>10</v>
+      </c>
+      <c r="W21" t="n">
+        <v>10</v>
+      </c>
+      <c r="X21" s="89" t="n"/>
+      <c r="Y21" s="41" t="n"/>
     </row>
     <row r="22" ht="19.5" customHeight="1" s="70">
       <c r="A22" s="90" t="n"/>
@@ -3514,8 +3614,14 @@
       <c r="U22" t="n">
         <v>10</v>
       </c>
-      <c r="V22" s="89" t="n"/>
-      <c r="W22" s="41" t="n"/>
+      <c r="V22" t="n">
+        <v>9</v>
+      </c>
+      <c r="W22" t="n">
+        <v>10</v>
+      </c>
+      <c r="X22" s="89" t="n"/>
+      <c r="Y22" s="41" t="n"/>
     </row>
     <row r="23" ht="19.5" customHeight="1" s="70">
       <c r="A23" s="90" t="n"/>
@@ -3569,8 +3675,14 @@
       <c r="U23" t="n">
         <v>10</v>
       </c>
-      <c r="V23" s="89" t="n"/>
-      <c r="W23" s="41" t="n"/>
+      <c r="V23" t="n">
+        <v>9</v>
+      </c>
+      <c r="W23" t="n">
+        <v>10</v>
+      </c>
+      <c r="X23" s="89" t="n"/>
+      <c r="Y23" s="41" t="n"/>
     </row>
     <row r="24" ht="19.5" customHeight="1" s="70">
       <c r="A24" s="90" t="n"/>
@@ -3624,8 +3736,14 @@
       <c r="U24" t="n">
         <v>10</v>
       </c>
-      <c r="V24" s="89" t="n"/>
-      <c r="W24" s="41" t="n"/>
+      <c r="V24" t="n">
+        <v>9</v>
+      </c>
+      <c r="W24" t="n">
+        <v>10</v>
+      </c>
+      <c r="X24" s="89" t="n"/>
+      <c r="Y24" s="41" t="n"/>
     </row>
     <row r="25" ht="19.5" customHeight="1" s="70">
       <c r="A25" s="88" t="n"/>
@@ -3679,8 +3797,14 @@
       <c r="U25" t="n">
         <v>10</v>
       </c>
-      <c r="V25" s="89" t="n"/>
-      <c r="W25" s="41" t="n"/>
+      <c r="V25" t="n">
+        <v>9</v>
+      </c>
+      <c r="W25" t="n">
+        <v>10</v>
+      </c>
+      <c r="X25" s="89" t="n"/>
+      <c r="Y25" s="41" t="n"/>
     </row>
     <row r="26" ht="19.5" customHeight="1" s="70">
       <c r="A26" s="48" t="inlineStr">
@@ -3744,8 +3868,14 @@
       <c r="U26" t="n">
         <v>10</v>
       </c>
-      <c r="V26" s="89" t="n"/>
-      <c r="W26" s="41" t="n"/>
+      <c r="V26" t="n">
+        <v>10</v>
+      </c>
+      <c r="W26" t="n">
+        <v>9</v>
+      </c>
+      <c r="X26" s="89" t="n"/>
+      <c r="Y26" s="41" t="n"/>
     </row>
     <row r="27" ht="19.5" customHeight="1" s="70">
       <c r="A27" s="90" t="n"/>
@@ -3799,8 +3929,14 @@
       <c r="U27" t="n">
         <v>9</v>
       </c>
-      <c r="V27" s="89" t="n"/>
-      <c r="W27" s="41" t="n"/>
+      <c r="V27" t="n">
+        <v>9</v>
+      </c>
+      <c r="W27" t="n">
+        <v>9</v>
+      </c>
+      <c r="X27" s="89" t="n"/>
+      <c r="Y27" s="41" t="n"/>
     </row>
     <row r="28" ht="19.5" customHeight="1" s="70">
       <c r="A28" s="90" t="n"/>
@@ -3854,8 +3990,14 @@
       <c r="U28" t="n">
         <v>10</v>
       </c>
-      <c r="V28" s="89" t="n"/>
-      <c r="W28" s="41" t="n"/>
+      <c r="V28" t="n">
+        <v>9</v>
+      </c>
+      <c r="W28" t="n">
+        <v>9</v>
+      </c>
+      <c r="X28" s="89" t="n"/>
+      <c r="Y28" s="41" t="n"/>
     </row>
     <row r="29" ht="19.5" customHeight="1" s="70">
       <c r="A29" s="90" t="n"/>
@@ -3909,8 +4051,14 @@
       <c r="U29" t="n">
         <v>10</v>
       </c>
-      <c r="V29" s="89" t="n"/>
-      <c r="W29" s="41" t="n"/>
+      <c r="V29" t="n">
+        <v>9</v>
+      </c>
+      <c r="W29" t="n">
+        <v>9</v>
+      </c>
+      <c r="X29" s="89" t="n"/>
+      <c r="Y29" s="41" t="n"/>
     </row>
     <row r="30" ht="19.5" customHeight="1" s="70">
       <c r="A30" s="90" t="n"/>
@@ -3964,8 +4112,14 @@
       <c r="U30" t="n">
         <v>9</v>
       </c>
-      <c r="V30" s="89" t="n"/>
-      <c r="W30" s="41" t="n"/>
+      <c r="V30" t="n">
+        <v>9</v>
+      </c>
+      <c r="W30" t="n">
+        <v>9</v>
+      </c>
+      <c r="X30" s="89" t="n"/>
+      <c r="Y30" s="41" t="n"/>
     </row>
     <row r="31" ht="19.5" customHeight="1" s="70">
       <c r="A31" s="90" t="n"/>
@@ -4024,8 +4178,14 @@
       <c r="U31" t="n">
         <v>10</v>
       </c>
-      <c r="V31" s="89" t="n"/>
-      <c r="W31" s="41" t="n"/>
+      <c r="V31" t="n">
+        <v>10</v>
+      </c>
+      <c r="W31" t="n">
+        <v>10</v>
+      </c>
+      <c r="X31" s="89" t="n"/>
+      <c r="Y31" s="41" t="n"/>
     </row>
     <row r="32" ht="19.5" customHeight="1" s="70">
       <c r="A32" s="90" t="n"/>
@@ -4079,8 +4239,14 @@
       <c r="U32" t="n">
         <v>10</v>
       </c>
-      <c r="V32" s="89" t="n"/>
-      <c r="W32" s="41" t="n"/>
+      <c r="V32" t="n">
+        <v>9</v>
+      </c>
+      <c r="W32" t="n">
+        <v>10</v>
+      </c>
+      <c r="X32" s="89" t="n"/>
+      <c r="Y32" s="41" t="n"/>
     </row>
     <row r="33" ht="19.5" customHeight="1" s="70">
       <c r="A33" s="90" t="n"/>
@@ -4134,8 +4300,14 @@
       <c r="U33" t="n">
         <v>10</v>
       </c>
-      <c r="V33" s="89" t="n"/>
-      <c r="W33" s="41" t="n"/>
+      <c r="V33" t="n">
+        <v>9</v>
+      </c>
+      <c r="W33" t="n">
+        <v>10</v>
+      </c>
+      <c r="X33" s="89" t="n"/>
+      <c r="Y33" s="41" t="n"/>
     </row>
     <row r="34" ht="19.5" customHeight="1" s="70">
       <c r="A34" s="90" t="n"/>
@@ -4189,8 +4361,14 @@
       <c r="U34" t="n">
         <v>10</v>
       </c>
-      <c r="V34" s="89" t="n"/>
-      <c r="W34" s="41" t="n"/>
+      <c r="V34" t="n">
+        <v>9</v>
+      </c>
+      <c r="W34" t="n">
+        <v>10</v>
+      </c>
+      <c r="X34" s="89" t="n"/>
+      <c r="Y34" s="41" t="n"/>
     </row>
     <row r="35" ht="19.5" customHeight="1" s="70">
       <c r="A35" s="88" t="n"/>
@@ -4244,8 +4422,14 @@
       <c r="U35" t="n">
         <v>10</v>
       </c>
-      <c r="V35" s="89" t="n"/>
-      <c r="W35" s="41" t="n"/>
+      <c r="V35" t="n">
+        <v>9</v>
+      </c>
+      <c r="W35" t="n">
+        <v>10</v>
+      </c>
+      <c r="X35" s="89" t="n"/>
+      <c r="Y35" s="41" t="n"/>
     </row>
     <row r="36" ht="19.5" customHeight="1" s="70">
       <c r="A36" s="48" t="inlineStr">
@@ -4309,8 +4493,14 @@
       <c r="U36" t="n">
         <v>10</v>
       </c>
-      <c r="V36" s="89" t="n"/>
-      <c r="W36" s="41" t="n"/>
+      <c r="V36" t="n">
+        <v>10</v>
+      </c>
+      <c r="W36" t="n">
+        <v>10</v>
+      </c>
+      <c r="X36" s="89" t="n"/>
+      <c r="Y36" s="41" t="n"/>
     </row>
     <row r="37" ht="19.5" customHeight="1" s="70">
       <c r="A37" s="90" t="n"/>
@@ -4364,8 +4554,14 @@
       <c r="U37" t="n">
         <v>10</v>
       </c>
-      <c r="V37" s="89" t="n"/>
-      <c r="W37" s="41" t="n"/>
+      <c r="V37" t="n">
+        <v>9</v>
+      </c>
+      <c r="W37" t="n">
+        <v>9</v>
+      </c>
+      <c r="X37" s="89" t="n"/>
+      <c r="Y37" s="41" t="n"/>
     </row>
     <row r="38" ht="19.5" customHeight="1" s="70">
       <c r="A38" s="90" t="n"/>
@@ -4419,8 +4615,14 @@
       <c r="U38" t="n">
         <v>10</v>
       </c>
-      <c r="V38" s="89" t="n"/>
-      <c r="W38" s="41" t="n"/>
+      <c r="V38" t="n">
+        <v>9</v>
+      </c>
+      <c r="W38" t="n">
+        <v>9</v>
+      </c>
+      <c r="X38" s="89" t="n"/>
+      <c r="Y38" s="41" t="n"/>
     </row>
     <row r="39" ht="19.5" customHeight="1" s="70">
       <c r="A39" s="90" t="n"/>
@@ -4474,8 +4676,14 @@
       <c r="U39" t="n">
         <v>10</v>
       </c>
-      <c r="V39" s="89" t="n"/>
-      <c r="W39" s="41" t="n"/>
+      <c r="V39" t="n">
+        <v>9</v>
+      </c>
+      <c r="W39" t="n">
+        <v>9</v>
+      </c>
+      <c r="X39" s="89" t="n"/>
+      <c r="Y39" s="41" t="n"/>
     </row>
     <row r="40" ht="19.5" customHeight="1" s="70">
       <c r="A40" s="90" t="n"/>
@@ -4529,8 +4737,14 @@
       <c r="U40" t="n">
         <v>10</v>
       </c>
-      <c r="V40" s="89" t="n"/>
-      <c r="W40" s="41" t="n"/>
+      <c r="V40" t="n">
+        <v>9</v>
+      </c>
+      <c r="W40" t="n">
+        <v>10</v>
+      </c>
+      <c r="X40" s="89" t="n"/>
+      <c r="Y40" s="41" t="n"/>
     </row>
     <row r="41" ht="19.5" customHeight="1" s="70">
       <c r="A41" s="90" t="n"/>
@@ -4589,8 +4803,14 @@
       <c r="U41" t="n">
         <v>9</v>
       </c>
-      <c r="V41" s="89" t="n"/>
-      <c r="W41" s="41" t="n"/>
+      <c r="V41" t="n">
+        <v>10</v>
+      </c>
+      <c r="W41" t="n">
+        <v>10</v>
+      </c>
+      <c r="X41" s="89" t="n"/>
+      <c r="Y41" s="41" t="n"/>
     </row>
     <row r="42" ht="19.5" customHeight="1" s="70">
       <c r="A42" s="90" t="n"/>
@@ -4644,8 +4864,14 @@
       <c r="U42" t="n">
         <v>9</v>
       </c>
-      <c r="V42" s="89" t="n"/>
-      <c r="W42" s="41" t="n"/>
+      <c r="V42" t="n">
+        <v>9</v>
+      </c>
+      <c r="W42" t="n">
+        <v>10</v>
+      </c>
+      <c r="X42" s="89" t="n"/>
+      <c r="Y42" s="41" t="n"/>
     </row>
     <row r="43" ht="19.5" customHeight="1" s="70">
       <c r="A43" s="90" t="n"/>
@@ -4699,8 +4925,14 @@
       <c r="U43" t="n">
         <v>9</v>
       </c>
-      <c r="V43" s="89" t="n"/>
-      <c r="W43" s="41" t="n"/>
+      <c r="V43" t="n">
+        <v>9</v>
+      </c>
+      <c r="W43" t="n">
+        <v>10</v>
+      </c>
+      <c r="X43" s="89" t="n"/>
+      <c r="Y43" s="41" t="n"/>
     </row>
     <row r="44" ht="19.5" customHeight="1" s="70">
       <c r="A44" s="90" t="n"/>
@@ -4754,8 +4986,14 @@
       <c r="U44" t="n">
         <v>9</v>
       </c>
-      <c r="V44" s="89" t="n"/>
-      <c r="W44" s="41" t="n"/>
+      <c r="V44" t="n">
+        <v>9</v>
+      </c>
+      <c r="W44" t="n">
+        <v>10</v>
+      </c>
+      <c r="X44" s="89" t="n"/>
+      <c r="Y44" s="41" t="n"/>
     </row>
     <row r="45" ht="19.5" customHeight="1" s="70">
       <c r="A45" s="88" t="n"/>
@@ -4809,8 +5047,14 @@
       <c r="U45" t="n">
         <v>9</v>
       </c>
-      <c r="V45" s="89" t="n"/>
-      <c r="W45" s="41" t="n"/>
+      <c r="V45" t="n">
+        <v>9</v>
+      </c>
+      <c r="W45" t="n">
+        <v>10</v>
+      </c>
+      <c r="X45" s="89" t="n"/>
+      <c r="Y45" s="41" t="n"/>
     </row>
     <row r="46" ht="19.5" customHeight="1" s="70">
       <c r="A46" s="48" t="inlineStr">
@@ -4874,8 +5118,14 @@
       <c r="U46" t="n">
         <v>10</v>
       </c>
-      <c r="V46" s="89" t="n"/>
-      <c r="W46" s="41" t="n"/>
+      <c r="V46" t="n">
+        <v>10</v>
+      </c>
+      <c r="W46" t="n">
+        <v>10</v>
+      </c>
+      <c r="X46" s="89" t="n"/>
+      <c r="Y46" s="41" t="n"/>
     </row>
     <row r="47" ht="19.5" customHeight="1" s="70">
       <c r="A47" s="90" t="n"/>
@@ -4929,8 +5179,14 @@
       <c r="U47" t="n">
         <v>10</v>
       </c>
-      <c r="V47" s="89" t="n"/>
-      <c r="W47" s="41" t="n"/>
+      <c r="V47" t="n">
+        <v>9</v>
+      </c>
+      <c r="W47" t="n">
+        <v>9</v>
+      </c>
+      <c r="X47" s="89" t="n"/>
+      <c r="Y47" s="41" t="n"/>
     </row>
     <row r="48" ht="19.5" customHeight="1" s="70">
       <c r="A48" s="90" t="n"/>
@@ -4984,8 +5240,14 @@
       <c r="U48" t="n">
         <v>10</v>
       </c>
-      <c r="V48" s="89" t="n"/>
-      <c r="W48" s="41" t="n"/>
+      <c r="V48" t="n">
+        <v>9</v>
+      </c>
+      <c r="W48" t="n">
+        <v>10</v>
+      </c>
+      <c r="X48" s="89" t="n"/>
+      <c r="Y48" s="41" t="n"/>
     </row>
     <row r="49" ht="19.5" customHeight="1" s="70">
       <c r="A49" s="90" t="n"/>
@@ -5039,8 +5301,14 @@
       <c r="U49" t="n">
         <v>10</v>
       </c>
-      <c r="V49" s="89" t="n"/>
-      <c r="W49" s="41" t="n"/>
+      <c r="V49" t="n">
+        <v>9</v>
+      </c>
+      <c r="W49" t="n">
+        <v>9</v>
+      </c>
+      <c r="X49" s="89" t="n"/>
+      <c r="Y49" s="41" t="n"/>
     </row>
     <row r="50" ht="19.5" customHeight="1" s="70">
       <c r="A50" s="90" t="n"/>
@@ -5094,8 +5362,14 @@
       <c r="U50" t="n">
         <v>10</v>
       </c>
-      <c r="V50" s="89" t="n"/>
-      <c r="W50" s="41" t="n"/>
+      <c r="V50" t="n">
+        <v>9</v>
+      </c>
+      <c r="W50" t="n">
+        <v>10</v>
+      </c>
+      <c r="X50" s="89" t="n"/>
+      <c r="Y50" s="41" t="n"/>
     </row>
     <row r="51" ht="19.5" customHeight="1" s="70">
       <c r="A51" s="90" t="n"/>
@@ -5154,8 +5428,14 @@
       <c r="U51" t="n">
         <v>10</v>
       </c>
-      <c r="V51" s="89" t="n"/>
-      <c r="W51" s="41" t="n"/>
+      <c r="V51" t="n">
+        <v>10</v>
+      </c>
+      <c r="W51" t="n">
+        <v>10</v>
+      </c>
+      <c r="X51" s="89" t="n"/>
+      <c r="Y51" s="41" t="n"/>
     </row>
     <row r="52" ht="19.5" customHeight="1" s="70">
       <c r="A52" s="90" t="n"/>
@@ -5209,8 +5489,14 @@
       <c r="U52" t="n">
         <v>10</v>
       </c>
-      <c r="V52" s="89" t="n"/>
-      <c r="W52" s="41" t="n"/>
+      <c r="V52" t="n">
+        <v>9</v>
+      </c>
+      <c r="W52" t="n">
+        <v>10</v>
+      </c>
+      <c r="X52" s="89" t="n"/>
+      <c r="Y52" s="41" t="n"/>
     </row>
     <row r="53" ht="19.5" customHeight="1" s="70">
       <c r="A53" s="90" t="n"/>
@@ -5264,8 +5550,14 @@
       <c r="U53" t="n">
         <v>10</v>
       </c>
-      <c r="V53" s="89" t="n"/>
-      <c r="W53" s="41" t="n"/>
+      <c r="V53" t="n">
+        <v>9</v>
+      </c>
+      <c r="W53" t="n">
+        <v>10</v>
+      </c>
+      <c r="X53" s="89" t="n"/>
+      <c r="Y53" s="41" t="n"/>
     </row>
     <row r="54" ht="19.5" customHeight="1" s="70">
       <c r="A54" s="90" t="n"/>
@@ -5319,8 +5611,14 @@
       <c r="U54" t="n">
         <v>10</v>
       </c>
-      <c r="V54" s="89" t="n"/>
-      <c r="W54" s="41" t="n"/>
+      <c r="V54" t="n">
+        <v>9</v>
+      </c>
+      <c r="W54" t="n">
+        <v>10</v>
+      </c>
+      <c r="X54" s="89" t="n"/>
+      <c r="Y54" s="41" t="n"/>
     </row>
     <row r="55" ht="19.5" customHeight="1" s="70">
       <c r="A55" s="90" t="n"/>
@@ -5374,8 +5672,14 @@
       <c r="U55" t="n">
         <v>10</v>
       </c>
-      <c r="V55" s="89" t="n"/>
-      <c r="W55" s="41" t="n"/>
+      <c r="V55" t="n">
+        <v>9</v>
+      </c>
+      <c r="W55" t="n">
+        <v>9</v>
+      </c>
+      <c r="X55" s="89" t="n"/>
+      <c r="Y55" s="41" t="n"/>
     </row>
     <row r="56" ht="20.25" customHeight="1" s="70">
       <c r="A56" s="90" t="n"/>
@@ -5403,8 +5707,8 @@
       <c r="N56" s="51" t="n"/>
       <c r="O56" s="51" t="n"/>
       <c r="P56" s="51" t="n"/>
-      <c r="V56" s="89" t="n"/>
-      <c r="W56" s="41" t="n"/>
+      <c r="X56" s="89" t="n"/>
+      <c r="Y56" s="41" t="n"/>
     </row>
     <row r="57" ht="20.25" customHeight="1" s="70">
       <c r="A57" s="90" t="n"/>
@@ -5427,8 +5731,8 @@
       <c r="N57" s="51" t="n"/>
       <c r="O57" s="51" t="n"/>
       <c r="P57" s="51" t="n"/>
-      <c r="V57" s="89" t="n"/>
-      <c r="W57" s="41" t="n"/>
+      <c r="X57" s="89" t="n"/>
+      <c r="Y57" s="41" t="n"/>
     </row>
     <row r="58" ht="20.25" customHeight="1" s="70">
       <c r="A58" s="90" t="n"/>
@@ -5451,8 +5755,8 @@
       <c r="N58" s="53" t="n"/>
       <c r="O58" s="53" t="n"/>
       <c r="P58" s="53" t="n"/>
-      <c r="V58" s="89" t="n"/>
-      <c r="W58" s="41" t="n"/>
+      <c r="X58" s="89" t="n"/>
+      <c r="Y58" s="41" t="n"/>
     </row>
     <row r="59" ht="20.25" customHeight="1" s="70">
       <c r="A59" s="88" t="n"/>
@@ -5475,8 +5779,8 @@
       <c r="N59" s="53" t="n"/>
       <c r="O59" s="53" t="n"/>
       <c r="P59" s="53" t="n"/>
-      <c r="V59" s="89" t="n"/>
-      <c r="W59" s="41" t="n"/>
+      <c r="X59" s="89" t="n"/>
+      <c r="Y59" s="41" t="n"/>
     </row>
     <row r="60" ht="20.25" customHeight="1" s="70">
       <c r="A60" s="48" t="inlineStr">
@@ -5541,8 +5845,14 @@
       <c r="U60" t="n">
         <v>10</v>
       </c>
-      <c r="V60" s="89" t="n"/>
-      <c r="W60" s="41" t="n"/>
+      <c r="V60" t="n">
+        <v>10</v>
+      </c>
+      <c r="W60" t="n">
+        <v>10</v>
+      </c>
+      <c r="X60" s="89" t="n"/>
+      <c r="Y60" s="41" t="n"/>
     </row>
     <row r="61" ht="20.25" customHeight="1" s="70">
       <c r="A61" s="90" t="n"/>
@@ -5556,7 +5866,7 @@
         <v>10</v>
       </c>
       <c r="E61" s="51" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F61" s="51" t="n">
         <v>9</v>
@@ -5596,8 +5906,14 @@
       <c r="U61" t="n">
         <v>10</v>
       </c>
-      <c r="V61" s="89" t="n"/>
-      <c r="W61" s="41" t="n"/>
+      <c r="V61" t="n">
+        <v>9</v>
+      </c>
+      <c r="W61" t="n">
+        <v>10</v>
+      </c>
+      <c r="X61" s="89" t="n"/>
+      <c r="Y61" s="41" t="n"/>
     </row>
     <row r="62" ht="20.25" customHeight="1" s="70">
       <c r="A62" s="90" t="n"/>
@@ -5611,7 +5927,7 @@
         <v>10</v>
       </c>
       <c r="E62" s="51" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F62" s="51" t="n">
         <v>9</v>
@@ -5651,8 +5967,14 @@
       <c r="U62" t="n">
         <v>10</v>
       </c>
-      <c r="V62" s="89" t="n"/>
-      <c r="W62" s="41" t="n"/>
+      <c r="V62" t="n">
+        <v>9</v>
+      </c>
+      <c r="W62" t="n">
+        <v>10</v>
+      </c>
+      <c r="X62" s="89" t="n"/>
+      <c r="Y62" s="41" t="n"/>
     </row>
     <row r="63" ht="20.25" customHeight="1" s="70">
       <c r="A63" s="90" t="n"/>
@@ -5698,7 +6020,7 @@
         <v>10</v>
       </c>
       <c r="S63" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="T63" t="n">
         <v>10</v>
@@ -5706,8 +6028,14 @@
       <c r="U63" t="n">
         <v>10</v>
       </c>
-      <c r="V63" s="89" t="n"/>
-      <c r="W63" s="41" t="n"/>
+      <c r="V63" t="n">
+        <v>9</v>
+      </c>
+      <c r="W63" t="n">
+        <v>10</v>
+      </c>
+      <c r="X63" s="89" t="n"/>
+      <c r="Y63" s="41" t="n"/>
     </row>
     <row r="64" ht="20.25" customHeight="1" s="70">
       <c r="A64" s="90" t="n"/>
@@ -5721,7 +6049,7 @@
         <v>10</v>
       </c>
       <c r="E64" s="55" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F64" s="55" t="n">
         <v>9</v>
@@ -5753,7 +6081,7 @@
         <v>10</v>
       </c>
       <c r="S64" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="T64" t="n">
         <v>10</v>
@@ -5761,8 +6089,14 @@
       <c r="U64" t="n">
         <v>10</v>
       </c>
-      <c r="V64" s="89" t="n"/>
-      <c r="W64" s="41" t="n"/>
+      <c r="V64" t="n">
+        <v>9</v>
+      </c>
+      <c r="W64" t="n">
+        <v>10</v>
+      </c>
+      <c r="X64" s="89" t="n"/>
+      <c r="Y64" s="41" t="n"/>
     </row>
     <row r="65" ht="20.25" customHeight="1" s="70">
       <c r="A65" s="90" t="n"/>
@@ -5778,21 +6112,52 @@
           <t>Course Contenet</t>
         </is>
       </c>
-      <c r="D65" s="51" t="n"/>
-      <c r="E65" s="51" t="n"/>
-      <c r="F65" s="51" t="n"/>
-      <c r="G65" s="51" t="n"/>
-      <c r="H65" s="51" t="n"/>
-      <c r="I65" s="51" t="n"/>
+      <c r="D65" s="51" t="n">
+        <v>10</v>
+      </c>
+      <c r="E65" s="51" t="n">
+        <v>9</v>
+      </c>
+      <c r="F65" s="51" t="n">
+        <v>9</v>
+      </c>
+      <c r="G65" s="51" t="n">
+        <v>10</v>
+      </c>
+      <c r="H65" s="51" t="n">
+        <v>9</v>
+      </c>
+      <c r="I65" s="51" t="n">
+        <v>9</v>
+      </c>
       <c r="J65" s="51" t="n"/>
-      <c r="K65" s="51" t="n"/>
-      <c r="L65" s="53" t="n"/>
+      <c r="K65" s="51" t="n">
+        <v>9</v>
+      </c>
+      <c r="L65" s="53" t="n">
+        <v>10</v>
+      </c>
       <c r="M65" s="51" t="n"/>
       <c r="N65" s="51" t="n"/>
       <c r="O65" s="51" t="n"/>
       <c r="P65" s="51" t="n"/>
-      <c r="V65" s="89" t="n"/>
-      <c r="W65" s="41" t="n"/>
+      <c r="S65" t="n">
+        <v>9</v>
+      </c>
+      <c r="T65" t="n">
+        <v>10</v>
+      </c>
+      <c r="U65" t="n">
+        <v>10</v>
+      </c>
+      <c r="V65" t="n">
+        <v>10</v>
+      </c>
+      <c r="W65" t="n">
+        <v>10</v>
+      </c>
+      <c r="X65" s="89" t="n"/>
+      <c r="Y65" s="41" t="n"/>
     </row>
     <row r="66" ht="20.25" customHeight="1" s="70">
       <c r="A66" s="90" t="n"/>
@@ -5802,21 +6167,52 @@
           <t>Structure &amp; Flow</t>
         </is>
       </c>
-      <c r="D66" s="51" t="n"/>
-      <c r="E66" s="51" t="n"/>
-      <c r="F66" s="51" t="n"/>
-      <c r="G66" s="51" t="n"/>
-      <c r="H66" s="51" t="n"/>
-      <c r="I66" s="51" t="n"/>
+      <c r="D66" s="51" t="n">
+        <v>10</v>
+      </c>
+      <c r="E66" s="51" t="n">
+        <v>9</v>
+      </c>
+      <c r="F66" s="51" t="n">
+        <v>9</v>
+      </c>
+      <c r="G66" s="51" t="n">
+        <v>10</v>
+      </c>
+      <c r="H66" s="51" t="n">
+        <v>9</v>
+      </c>
+      <c r="I66" s="51" t="n">
+        <v>9</v>
+      </c>
       <c r="J66" s="51" t="n"/>
-      <c r="K66" s="51" t="n"/>
-      <c r="L66" s="53" t="n"/>
+      <c r="K66" s="51" t="n">
+        <v>9</v>
+      </c>
+      <c r="L66" s="53" t="n">
+        <v>10</v>
+      </c>
       <c r="M66" s="51" t="n"/>
       <c r="N66" s="51" t="n"/>
       <c r="O66" s="51" t="n"/>
       <c r="P66" s="51" t="n"/>
-      <c r="V66" s="89" t="n"/>
-      <c r="W66" s="41" t="n"/>
+      <c r="S66" t="n">
+        <v>9</v>
+      </c>
+      <c r="T66" t="n">
+        <v>10</v>
+      </c>
+      <c r="U66" t="n">
+        <v>10</v>
+      </c>
+      <c r="V66" t="n">
+        <v>9</v>
+      </c>
+      <c r="W66" t="n">
+        <v>10</v>
+      </c>
+      <c r="X66" s="89" t="n"/>
+      <c r="Y66" s="41" t="n"/>
     </row>
     <row r="67" ht="20.25" customHeight="1" s="70">
       <c r="A67" s="90" t="n"/>
@@ -5826,21 +6222,52 @@
           <t>Time Management</t>
         </is>
       </c>
-      <c r="D67" s="51" t="n"/>
-      <c r="E67" s="51" t="n"/>
-      <c r="F67" s="51" t="n"/>
-      <c r="G67" s="51" t="n"/>
-      <c r="H67" s="51" t="n"/>
-      <c r="I67" s="51" t="n"/>
+      <c r="D67" s="51" t="n">
+        <v>10</v>
+      </c>
+      <c r="E67" s="51" t="n">
+        <v>9</v>
+      </c>
+      <c r="F67" s="51" t="n">
+        <v>9</v>
+      </c>
+      <c r="G67" s="51" t="n">
+        <v>10</v>
+      </c>
+      <c r="H67" s="51" t="n">
+        <v>9</v>
+      </c>
+      <c r="I67" s="51" t="n">
+        <v>9</v>
+      </c>
       <c r="J67" s="51" t="n"/>
-      <c r="K67" s="51" t="n"/>
-      <c r="L67" s="53" t="n"/>
+      <c r="K67" s="51" t="n">
+        <v>9</v>
+      </c>
+      <c r="L67" s="53" t="n">
+        <v>10</v>
+      </c>
       <c r="M67" s="51" t="n"/>
       <c r="N67" s="51" t="n"/>
       <c r="O67" s="51" t="n"/>
       <c r="P67" s="51" t="n"/>
-      <c r="V67" s="89" t="n"/>
-      <c r="W67" s="41" t="n"/>
+      <c r="S67" t="n">
+        <v>9</v>
+      </c>
+      <c r="T67" t="n">
+        <v>10</v>
+      </c>
+      <c r="U67" t="n">
+        <v>10</v>
+      </c>
+      <c r="V67" t="n">
+        <v>9</v>
+      </c>
+      <c r="W67" t="n">
+        <v>10</v>
+      </c>
+      <c r="X67" s="89" t="n"/>
+      <c r="Y67" s="41" t="n"/>
     </row>
     <row r="68" ht="20.25" customHeight="1" s="70">
       <c r="A68" s="90" t="n"/>
@@ -5850,21 +6277,52 @@
           <t>Faculty Delivery</t>
         </is>
       </c>
-      <c r="D68" s="53" t="n"/>
-      <c r="E68" s="53" t="n"/>
-      <c r="F68" s="53" t="n"/>
-      <c r="G68" s="53" t="n"/>
-      <c r="H68" s="51" t="n"/>
-      <c r="I68" s="53" t="n"/>
+      <c r="D68" s="53" t="n">
+        <v>10</v>
+      </c>
+      <c r="E68" s="53" t="n">
+        <v>9</v>
+      </c>
+      <c r="F68" s="53" t="n">
+        <v>9</v>
+      </c>
+      <c r="G68" s="53" t="n">
+        <v>10</v>
+      </c>
+      <c r="H68" s="51" t="n">
+        <v>9</v>
+      </c>
+      <c r="I68" s="53" t="n">
+        <v>9</v>
+      </c>
       <c r="J68" s="53" t="n"/>
-      <c r="K68" s="53" t="n"/>
-      <c r="L68" s="53" t="n"/>
+      <c r="K68" s="53" t="n">
+        <v>9</v>
+      </c>
+      <c r="L68" s="53" t="n">
+        <v>10</v>
+      </c>
       <c r="M68" s="53" t="n"/>
       <c r="N68" s="53" t="n"/>
       <c r="O68" s="53" t="n"/>
       <c r="P68" s="53" t="n"/>
-      <c r="V68" s="89" t="n"/>
-      <c r="W68" s="41" t="n"/>
+      <c r="S68" t="n">
+        <v>9</v>
+      </c>
+      <c r="T68" t="n">
+        <v>10</v>
+      </c>
+      <c r="U68" t="n">
+        <v>10</v>
+      </c>
+      <c r="V68" t="n">
+        <v>9</v>
+      </c>
+      <c r="W68" t="n">
+        <v>10</v>
+      </c>
+      <c r="X68" s="89" t="n"/>
+      <c r="Y68" s="41" t="n"/>
     </row>
     <row r="69" ht="20.25" customHeight="1" s="70">
       <c r="A69" s="90" t="n"/>
@@ -5874,21 +6332,52 @@
           <t>Faculty Participants Interaction</t>
         </is>
       </c>
-      <c r="D69" s="55" t="n"/>
-      <c r="E69" s="55" t="n"/>
-      <c r="F69" s="55" t="n"/>
-      <c r="G69" s="55" t="n"/>
-      <c r="H69" s="51" t="n"/>
-      <c r="I69" s="55" t="n"/>
+      <c r="D69" s="55" t="n">
+        <v>10</v>
+      </c>
+      <c r="E69" s="55" t="n">
+        <v>9</v>
+      </c>
+      <c r="F69" s="55" t="n">
+        <v>9</v>
+      </c>
+      <c r="G69" s="55" t="n">
+        <v>10</v>
+      </c>
+      <c r="H69" s="51" t="n">
+        <v>9</v>
+      </c>
+      <c r="I69" s="55" t="n">
+        <v>9</v>
+      </c>
       <c r="J69" s="55" t="n"/>
-      <c r="K69" s="55" t="n"/>
-      <c r="L69" s="53" t="n"/>
+      <c r="K69" s="55" t="n">
+        <v>9</v>
+      </c>
+      <c r="L69" s="53" t="n">
+        <v>10</v>
+      </c>
       <c r="M69" s="55" t="n"/>
       <c r="N69" s="55" t="n"/>
       <c r="O69" s="55" t="n"/>
       <c r="P69" s="55" t="n"/>
-      <c r="V69" s="89" t="n"/>
-      <c r="W69" s="41" t="n"/>
+      <c r="S69" t="n">
+        <v>9</v>
+      </c>
+      <c r="T69" t="n">
+        <v>10</v>
+      </c>
+      <c r="U69" t="n">
+        <v>10</v>
+      </c>
+      <c r="V69" t="n">
+        <v>9</v>
+      </c>
+      <c r="W69" t="n">
+        <v>10</v>
+      </c>
+      <c r="X69" s="89" t="n"/>
+      <c r="Y69" s="41" t="n"/>
     </row>
     <row r="70" ht="20.25" customHeight="1" s="70">
       <c r="A70" s="90" t="n"/>
@@ -5904,21 +6393,52 @@
           <t>Course Contenet</t>
         </is>
       </c>
-      <c r="D70" s="51" t="n"/>
-      <c r="E70" s="51" t="n"/>
-      <c r="F70" s="51" t="n"/>
-      <c r="G70" s="55" t="n"/>
-      <c r="H70" s="51" t="n"/>
-      <c r="I70" s="51" t="n"/>
+      <c r="D70" s="51" t="n">
+        <v>10</v>
+      </c>
+      <c r="E70" s="51" t="n">
+        <v>9</v>
+      </c>
+      <c r="F70" s="51" t="n">
+        <v>9</v>
+      </c>
+      <c r="G70" s="55" t="n">
+        <v>10</v>
+      </c>
+      <c r="H70" s="51" t="n">
+        <v>9</v>
+      </c>
+      <c r="I70" s="51" t="n">
+        <v>9</v>
+      </c>
       <c r="J70" s="51" t="n"/>
-      <c r="K70" s="51" t="n"/>
-      <c r="L70" s="53" t="n"/>
+      <c r="K70" s="51" t="n">
+        <v>9</v>
+      </c>
+      <c r="L70" s="53" t="n">
+        <v>10</v>
+      </c>
       <c r="M70" s="51" t="n"/>
       <c r="N70" s="51" t="n"/>
       <c r="O70" s="51" t="n"/>
       <c r="P70" s="51" t="n"/>
-      <c r="V70" s="89" t="n"/>
-      <c r="W70" s="41" t="n"/>
+      <c r="S70" t="n">
+        <v>9</v>
+      </c>
+      <c r="T70" t="n">
+        <v>10</v>
+      </c>
+      <c r="U70" t="n">
+        <v>10</v>
+      </c>
+      <c r="V70" t="n">
+        <v>10</v>
+      </c>
+      <c r="W70" t="n">
+        <v>10</v>
+      </c>
+      <c r="X70" s="89" t="n"/>
+      <c r="Y70" s="41" t="n"/>
     </row>
     <row r="71" ht="20.25" customHeight="1" s="70">
       <c r="A71" s="90" t="n"/>
@@ -5928,21 +6448,52 @@
           <t>Structure &amp; Flow</t>
         </is>
       </c>
-      <c r="D71" s="51" t="n"/>
-      <c r="E71" s="51" t="n"/>
-      <c r="F71" s="51" t="n"/>
-      <c r="G71" s="55" t="n"/>
-      <c r="H71" s="51" t="n"/>
-      <c r="I71" s="51" t="n"/>
+      <c r="D71" s="51" t="n">
+        <v>10</v>
+      </c>
+      <c r="E71" s="51" t="n">
+        <v>8</v>
+      </c>
+      <c r="F71" s="51" t="n">
+        <v>9</v>
+      </c>
+      <c r="G71" s="55" t="n">
+        <v>10</v>
+      </c>
+      <c r="H71" s="51" t="n">
+        <v>9</v>
+      </c>
+      <c r="I71" s="51" t="n">
+        <v>9</v>
+      </c>
       <c r="J71" s="51" t="n"/>
-      <c r="K71" s="51" t="n"/>
-      <c r="L71" s="53" t="n"/>
+      <c r="K71" s="51" t="n">
+        <v>9</v>
+      </c>
+      <c r="L71" s="53" t="n">
+        <v>10</v>
+      </c>
       <c r="M71" s="51" t="n"/>
       <c r="N71" s="51" t="n"/>
       <c r="O71" s="51" t="n"/>
       <c r="P71" s="51" t="n"/>
-      <c r="V71" s="89" t="n"/>
-      <c r="W71" s="41" t="n"/>
+      <c r="S71" t="n">
+        <v>9</v>
+      </c>
+      <c r="T71" t="n">
+        <v>10</v>
+      </c>
+      <c r="U71" t="n">
+        <v>10</v>
+      </c>
+      <c r="V71" t="n">
+        <v>9</v>
+      </c>
+      <c r="W71" t="n">
+        <v>10</v>
+      </c>
+      <c r="X71" s="89" t="n"/>
+      <c r="Y71" s="41" t="n"/>
     </row>
     <row r="72" ht="20.25" customHeight="1" s="70">
       <c r="A72" s="90" t="n"/>
@@ -5952,21 +6503,52 @@
           <t>Time Management</t>
         </is>
       </c>
-      <c r="D72" s="51" t="n"/>
-      <c r="E72" s="51" t="n"/>
-      <c r="F72" s="51" t="n"/>
-      <c r="G72" s="55" t="n"/>
-      <c r="H72" s="51" t="n"/>
-      <c r="I72" s="51" t="n"/>
+      <c r="D72" s="51" t="n">
+        <v>10</v>
+      </c>
+      <c r="E72" s="51" t="n">
+        <v>9</v>
+      </c>
+      <c r="F72" s="51" t="n">
+        <v>9</v>
+      </c>
+      <c r="G72" s="55" t="n">
+        <v>10</v>
+      </c>
+      <c r="H72" s="51" t="n">
+        <v>9</v>
+      </c>
+      <c r="I72" s="51" t="n">
+        <v>9</v>
+      </c>
       <c r="J72" s="51" t="n"/>
-      <c r="K72" s="51" t="n"/>
-      <c r="L72" s="53" t="n"/>
+      <c r="K72" s="51" t="n">
+        <v>9</v>
+      </c>
+      <c r="L72" s="53" t="n">
+        <v>10</v>
+      </c>
       <c r="M72" s="51" t="n"/>
       <c r="N72" s="51" t="n"/>
       <c r="O72" s="51" t="n"/>
       <c r="P72" s="51" t="n"/>
-      <c r="V72" s="89" t="n"/>
-      <c r="W72" s="41" t="n"/>
+      <c r="S72" t="n">
+        <v>9</v>
+      </c>
+      <c r="T72" t="n">
+        <v>10</v>
+      </c>
+      <c r="U72" t="n">
+        <v>10</v>
+      </c>
+      <c r="V72" t="n">
+        <v>9</v>
+      </c>
+      <c r="W72" t="n">
+        <v>10</v>
+      </c>
+      <c r="X72" s="89" t="n"/>
+      <c r="Y72" s="41" t="n"/>
     </row>
     <row r="73" ht="20.25" customHeight="1" s="70">
       <c r="A73" s="90" t="n"/>
@@ -5976,21 +6558,52 @@
           <t>Faculty Delivery</t>
         </is>
       </c>
-      <c r="D73" s="53" t="n"/>
-      <c r="E73" s="53" t="n"/>
-      <c r="F73" s="53" t="n"/>
-      <c r="G73" s="55" t="n"/>
-      <c r="H73" s="51" t="n"/>
-      <c r="I73" s="53" t="n"/>
+      <c r="D73" s="53" t="n">
+        <v>10</v>
+      </c>
+      <c r="E73" s="53" t="n">
+        <v>9</v>
+      </c>
+      <c r="F73" s="53" t="n">
+        <v>9</v>
+      </c>
+      <c r="G73" s="55" t="n">
+        <v>10</v>
+      </c>
+      <c r="H73" s="51" t="n">
+        <v>9</v>
+      </c>
+      <c r="I73" s="53" t="n">
+        <v>9</v>
+      </c>
       <c r="J73" s="53" t="n"/>
-      <c r="K73" s="53" t="n"/>
-      <c r="L73" s="53" t="n"/>
+      <c r="K73" s="53" t="n">
+        <v>9</v>
+      </c>
+      <c r="L73" s="53" t="n">
+        <v>10</v>
+      </c>
       <c r="M73" s="53" t="n"/>
       <c r="N73" s="53" t="n"/>
       <c r="O73" s="53" t="n"/>
       <c r="P73" s="53" t="n"/>
-      <c r="V73" s="89" t="n"/>
-      <c r="W73" s="41" t="n"/>
+      <c r="S73" t="n">
+        <v>9</v>
+      </c>
+      <c r="T73" t="n">
+        <v>10</v>
+      </c>
+      <c r="U73" t="n">
+        <v>10</v>
+      </c>
+      <c r="V73" t="n">
+        <v>10</v>
+      </c>
+      <c r="W73" t="n">
+        <v>10</v>
+      </c>
+      <c r="X73" s="89" t="n"/>
+      <c r="Y73" s="41" t="n"/>
     </row>
     <row r="74" ht="20.25" customHeight="1" s="70">
       <c r="A74" s="88" t="n"/>
@@ -6000,21 +6613,52 @@
           <t>Faculty Participants Interaction</t>
         </is>
       </c>
-      <c r="D74" s="55" t="n"/>
-      <c r="E74" s="55" t="n"/>
-      <c r="F74" s="55" t="n"/>
-      <c r="G74" s="55" t="n"/>
-      <c r="H74" s="51" t="n"/>
-      <c r="I74" s="55" t="n"/>
+      <c r="D74" s="55" t="n">
+        <v>10</v>
+      </c>
+      <c r="E74" s="55" t="n">
+        <v>10</v>
+      </c>
+      <c r="F74" s="55" t="n">
+        <v>9</v>
+      </c>
+      <c r="G74" s="55" t="n">
+        <v>10</v>
+      </c>
+      <c r="H74" s="51" t="n">
+        <v>9</v>
+      </c>
+      <c r="I74" s="55" t="n">
+        <v>9</v>
+      </c>
       <c r="J74" s="55" t="n"/>
-      <c r="K74" s="55" t="n"/>
-      <c r="L74" s="53" t="n"/>
+      <c r="K74" s="55" t="n">
+        <v>9</v>
+      </c>
+      <c r="L74" s="53" t="n">
+        <v>10</v>
+      </c>
       <c r="M74" s="55" t="n"/>
       <c r="N74" s="55" t="n"/>
       <c r="O74" s="55" t="n"/>
       <c r="P74" s="55" t="n"/>
-      <c r="V74" s="89" t="n"/>
-      <c r="W74" s="41" t="n"/>
+      <c r="S74" t="n">
+        <v>9</v>
+      </c>
+      <c r="T74" t="n">
+        <v>10</v>
+      </c>
+      <c r="U74" t="n">
+        <v>10</v>
+      </c>
+      <c r="V74" t="n">
+        <v>9</v>
+      </c>
+      <c r="W74" t="n">
+        <v>10</v>
+      </c>
+      <c r="X74" s="89" t="n"/>
+      <c r="Y74" s="41" t="n"/>
     </row>
     <row r="75" ht="20.25" customHeight="1" s="70">
       <c r="A75" s="61" t="inlineStr">
@@ -6072,8 +6716,14 @@
       <c r="U75" t="n">
         <v>9</v>
       </c>
-      <c r="V75" s="89" t="n"/>
-      <c r="W75" s="62" t="n"/>
+      <c r="V75" t="n">
+        <v>10</v>
+      </c>
+      <c r="W75" t="n">
+        <v>10</v>
+      </c>
+      <c r="X75" s="89" t="n"/>
+      <c r="Y75" s="62" t="n"/>
     </row>
     <row r="76" ht="20.25" customHeight="1" s="70">
       <c r="A76" s="92" t="n"/>
@@ -6127,8 +6777,14 @@
       <c r="U76" t="n">
         <v>9</v>
       </c>
-      <c r="V76" s="89" t="n"/>
-      <c r="W76" s="62" t="n"/>
+      <c r="V76" t="n">
+        <v>10</v>
+      </c>
+      <c r="W76" t="n">
+        <v>9</v>
+      </c>
+      <c r="X76" s="89" t="n"/>
+      <c r="Y76" s="62" t="n"/>
     </row>
     <row r="77" ht="20.25" customHeight="1" s="70">
       <c r="A77" s="92" t="n"/>
@@ -6182,8 +6838,14 @@
       <c r="U77" t="n">
         <v>9</v>
       </c>
-      <c r="V77" s="89" t="n"/>
-      <c r="W77" s="62" t="n"/>
+      <c r="V77" t="n">
+        <v>10</v>
+      </c>
+      <c r="W77" t="n">
+        <v>10</v>
+      </c>
+      <c r="X77" s="89" t="n"/>
+      <c r="Y77" s="62" t="n"/>
     </row>
     <row r="78" ht="20.25" customHeight="1" s="70">
       <c r="A78" s="94" t="n"/>
@@ -6237,8 +6899,14 @@
       <c r="U78" t="n">
         <v>9</v>
       </c>
-      <c r="V78" s="89" t="n"/>
-      <c r="W78" s="62" t="n"/>
+      <c r="V78" t="n">
+        <v>10</v>
+      </c>
+      <c r="W78" t="n">
+        <v>9</v>
+      </c>
+      <c r="X78" s="89" t="n"/>
+      <c r="Y78" s="62" t="n"/>
     </row>
     <row r="79" ht="59.25" customHeight="1" s="70">
       <c r="A79" s="61" t="inlineStr">
@@ -6261,8 +6929,8 @@
       <c r="N79" s="64" t="n"/>
       <c r="O79" s="66" t="n"/>
       <c r="P79" s="65" t="n"/>
-      <c r="V79" s="96" t="n"/>
-      <c r="W79" s="68" t="n"/>
+      <c r="X79" s="96" t="n"/>
+      <c r="Y79" s="68" t="n"/>
     </row>
     <row r="80" ht="55.5" customHeight="1" s="70">
       <c r="A80" s="61" t="inlineStr">
@@ -6285,8 +6953,8 @@
       <c r="N80" s="64" t="n"/>
       <c r="O80" s="64" t="n"/>
       <c r="P80" s="64" t="n"/>
-      <c r="V80" s="96" t="n"/>
-      <c r="W80" s="68" t="n"/>
+      <c r="X80" s="96" t="n"/>
+      <c r="Y80" s="68" t="n"/>
     </row>
     <row r="81" ht="15.75" customHeight="1" s="70">
       <c r="E81" s="69" t="n"/>

</xml_diff>